<commit_message>
Checkpoint: Se reemplazó la plantilla anterior por FORMATOREPORTEDEHERRAMIENTADAÑADA.pdf-1.xlsx. El reporte conserva la estructura recibida, coloca la descripción del evento completa en el bloque izquierdo y coloca las fotos reales cargadas en el bloque derecho de evidencias, sin textos genéricos que alteren el formato. Se validaron 13 pruebas, TypeScript, build y una prueba específica de la plantilla.
</commit_message>
<xml_diff>
--- a/server/templates/formato-herramienta-danada.xlsx
+++ b/server/templates/formato-herramienta-danada.xlsx
@@ -295,20 +295,16 @@
       <xdr:row>17</xdr:row>
       <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4514850" cy="1962150"/>
-    <xdr:sp macro="" textlink="">
+    <xdr:ext cx="4514850" cy="1676400"/>
+    <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="16" name="CuadroTexto 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}"/>
-          </a:extLst>
-        </xdr:cNvPr>
+        <xdr:cNvPr id="16" name="CuadroTexto 4"/>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3495675" y="3914775"/>
-          <a:ext cx="3924300" cy="1861185"/>
+          <a:off x="3904615" y="3276600"/>
+          <a:ext cx="4527550" cy="1680210"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -461,6 +457,7 @@
             <a:rPr lang="es-PE" sz="1400"/>
             <a:t> </a:t>
           </a:r>
+          <a:endParaRPr lang="es-PE" sz="1400"/>
         </a:p>
         <a:p>
           <a:pPr lvl="0" algn="l"/>
@@ -493,7 +490,7 @@
       <xdr:row>1</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2057400" cy="457200"/>
+    <xdr:ext cx="2057400" cy="428625"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="0" name="image1.png"/>
@@ -521,7 +518,7 @@
       <xdr:row>1</xdr:row>
       <xdr:rowOff>247650</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1114425" cy="962025"/>
+    <xdr:ext cx="1114425" cy="847725"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="0" name="image2.png"/>
@@ -529,62 +526,6 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="971550" cy="2667000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1095375</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1200150" cy="2486025"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -644,7 +585,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -677,26 +618,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -729,23 +653,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -907,10 +814,6 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}"/>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -927,10 +830,10 @@
     <col customWidth="1" min="6" max="6" width="11.25"/>
     <col customWidth="1" min="7" max="7" width="17.88"/>
     <col customWidth="1" min="8" max="9" width="11.38"/>
-    <col customWidth="1" min="10" max="11" width="10.63"/>
+    <col customWidth="1" min="10" max="11" width="11.0"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13.5" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="C1" s="3" t="s">
@@ -960,7 +863,7 @@
       <c r="J2" s="8"/>
       <c r="K2" s="8"/>
     </row>
-    <row r="3">
+    <row r="3" ht="13.5" customHeight="1">
       <c r="A3" s="9"/>
       <c r="B3" s="10"/>
       <c r="C3" s="12" t="s">
@@ -974,7 +877,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
     </row>
-    <row r="4">
+    <row r="4" ht="13.5" customHeight="1">
       <c r="A4" s="13"/>
       <c r="B4" s="15"/>
       <c r="C4" s="16" t="s">
@@ -988,7 +891,7 @@
       <c r="J4" s="8"/>
       <c r="K4" s="8"/>
     </row>
-    <row r="5">
+    <row r="5" ht="13.5" customHeight="1">
       <c r="A5" s="18" t="s">
         <v>5</v>
       </c>
@@ -1002,7 +905,7 @@
       <c r="J5" s="8"/>
       <c r="K5" s="8"/>
     </row>
-    <row r="6">
+    <row r="6" ht="13.5" customHeight="1">
       <c r="A6" s="18" t="s">
         <v>6</v>
       </c>
@@ -1016,7 +919,7 @@
       <c r="J6" s="8"/>
       <c r="K6" s="8"/>
     </row>
-    <row r="7">
+    <row r="7" ht="13.5" customHeight="1">
       <c r="A7" s="18" t="s">
         <v>7</v>
       </c>
@@ -1045,7 +948,7 @@
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
     </row>
-    <row r="9">
+    <row r="9" ht="13.5" customHeight="1">
       <c r="A9" s="21" t="s">
         <v>9</v>
       </c>
@@ -1060,7 +963,7 @@
       <c r="J9" s="8"/>
       <c r="K9" s="8"/>
     </row>
-    <row r="10">
+    <row r="10" ht="13.5" customHeight="1">
       <c r="A10" s="3" t="s">
         <v>10</v>
       </c>
@@ -1077,7 +980,7 @@
       <c r="J10" s="8"/>
       <c r="K10" s="8"/>
     </row>
-    <row r="11">
+    <row r="11" ht="13.5" customHeight="1">
       <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
@@ -1094,7 +997,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="8"/>
     </row>
-    <row r="12">
+    <row r="12" ht="13.5" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
@@ -1109,7 +1012,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="8"/>
     </row>
-    <row r="13">
+    <row r="13" ht="13.5" customHeight="1">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
@@ -1126,7 +1029,7 @@
       <c r="J13" s="8"/>
       <c r="K13" s="8"/>
     </row>
-    <row r="14">
+    <row r="14" ht="13.5" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>16</v>
       </c>
@@ -1141,7 +1044,7 @@
       <c r="J14" s="8"/>
       <c r="K14" s="8"/>
     </row>
-    <row r="15">
+    <row r="15" ht="13.5" customHeight="1">
       <c r="A15" s="3" t="s">
         <v>17</v>
       </c>
@@ -1156,7 +1059,7 @@
       <c r="J15" s="8"/>
       <c r="K15" s="8"/>
     </row>
-    <row r="16">
+    <row r="16" ht="13.5" customHeight="1">
       <c r="A16" s="21" t="s">
         <v>18</v>
       </c>
@@ -1171,7 +1074,7 @@
       <c r="J16" s="8"/>
       <c r="K16" s="8"/>
     </row>
-    <row r="17">
+    <row r="17" ht="13.5" customHeight="1">
       <c r="A17" s="1"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1184,79 +1087,79 @@
       <c r="J17" s="8"/>
       <c r="K17" s="8"/>
     </row>
-    <row r="18">
+    <row r="18" ht="13.5" customHeight="1">
       <c r="A18" s="9"/>
       <c r="I18" s="10"/>
       <c r="J18" s="8"/>
       <c r="K18" s="8"/>
     </row>
-    <row r="19">
+    <row r="19" ht="13.5" customHeight="1">
       <c r="A19" s="9"/>
       <c r="I19" s="10"/>
       <c r="J19" s="8"/>
       <c r="K19" s="8"/>
     </row>
-    <row r="20">
+    <row r="20" ht="13.5" customHeight="1">
       <c r="A20" s="9"/>
       <c r="I20" s="10"/>
       <c r="J20" s="8"/>
       <c r="K20" s="8"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21" ht="13.5" customHeight="1">
       <c r="A21" s="9"/>
       <c r="I21" s="10"/>
       <c r="J21" s="8"/>
       <c r="K21" s="8"/>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="22" ht="13.5" customHeight="1">
       <c r="A22" s="9"/>
       <c r="I22" s="10"/>
       <c r="J22" s="8"/>
       <c r="K22" s="8"/>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" ht="13.5" customHeight="1">
       <c r="A23" s="9"/>
       <c r="I23" s="10"/>
       <c r="J23" s="8"/>
       <c r="K23" s="8"/>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
+    <row r="24" ht="13.5" customHeight="1">
       <c r="A24" s="9"/>
       <c r="I24" s="10"/>
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
+    <row r="25" ht="13.5" customHeight="1">
       <c r="A25" s="9"/>
       <c r="I25" s="10"/>
       <c r="J25" s="8"/>
       <c r="K25" s="8"/>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
+    <row r="26" ht="13.5" customHeight="1">
       <c r="A26" s="9"/>
       <c r="I26" s="10"/>
       <c r="J26" s="8"/>
       <c r="K26" s="8"/>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
+    <row r="27" ht="13.5" customHeight="1">
       <c r="A27" s="9"/>
       <c r="I27" s="10"/>
       <c r="J27" s="8"/>
       <c r="K27" s="8"/>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
+    <row r="28" ht="13.5" customHeight="1">
       <c r="A28" s="9"/>
       <c r="I28" s="10"/>
       <c r="J28" s="8"/>
       <c r="K28" s="8"/>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
+    <row r="29" ht="13.5" customHeight="1">
       <c r="A29" s="9"/>
       <c r="I29" s="10"/>
       <c r="J29" s="8"/>
       <c r="K29" s="8"/>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
+    <row r="30" ht="13.5" customHeight="1">
       <c r="A30" s="13"/>
       <c r="B30" s="14"/>
       <c r="C30" s="14"/>
@@ -1269,7 +1172,7 @@
       <c r="J30" s="8"/>
       <c r="K30" s="8"/>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
+    <row r="31" ht="13.5" customHeight="1">
       <c r="A31" s="22"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
@@ -1282,13 +1185,13 @@
       <c r="J31" s="8"/>
       <c r="K31" s="8"/>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
+    <row r="32" ht="13.5" customHeight="1">
       <c r="A32" s="9"/>
       <c r="I32" s="10"/>
       <c r="J32" s="8"/>
       <c r="K32" s="8"/>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
+    <row r="33" ht="13.5" customHeight="1">
       <c r="A33" s="13"/>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -1301,7 +1204,7 @@
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
     </row>
-    <row r="34" ht="15.75" customHeight="1">
+    <row r="34" ht="13.5" customHeight="1">
       <c r="A34" s="23" t="s">
         <v>19</v>
       </c>
@@ -1316,7 +1219,7 @@
       <c r="J34" s="8"/>
       <c r="K34" s="8"/>
     </row>
-    <row r="35" ht="15.75" customHeight="1">
+    <row r="35" ht="13.5" customHeight="1">
       <c r="A35" s="1"/>
       <c r="B35" s="6"/>
       <c r="C35" s="2"/>
@@ -1329,7 +1232,7 @@
       <c r="J35" s="8"/>
       <c r="K35" s="8"/>
     </row>
-    <row r="36" ht="15.75" customHeight="1">
+    <row r="36" ht="13.5" customHeight="1">
       <c r="A36" s="9"/>
       <c r="C36" s="10"/>
       <c r="D36" s="9"/>
@@ -1339,7 +1242,7 @@
       <c r="J36" s="8"/>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
+    <row r="37" ht="13.5" customHeight="1">
       <c r="A37" s="9"/>
       <c r="C37" s="10"/>
       <c r="D37" s="9"/>
@@ -1349,7 +1252,7 @@
       <c r="J37" s="8"/>
       <c r="K37" s="8"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1">
+    <row r="38" ht="13.5" customHeight="1">
       <c r="A38" s="9"/>
       <c r="C38" s="10"/>
       <c r="D38" s="9"/>
@@ -1359,7 +1262,7 @@
       <c r="J38" s="8"/>
       <c r="K38" s="8"/>
     </row>
-    <row r="39" ht="15.75" customHeight="1">
+    <row r="39" ht="13.5" customHeight="1">
       <c r="A39" s="13"/>
       <c r="B39" s="14"/>
       <c r="C39" s="15"/>
@@ -1391,7 +1294,7 @@
       <c r="J40" s="8"/>
       <c r="K40" s="8"/>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
+    <row r="41" ht="13.5" customHeight="1">
       <c r="A41" s="8"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
@@ -1404,7 +1307,7 @@
       <c r="J41" s="8"/>
       <c r="K41" s="8"/>
     </row>
-    <row r="42" ht="15.75" customHeight="1">
+    <row r="42" ht="13.5" customHeight="1">
       <c r="A42" s="8"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
@@ -1417,7 +1320,7 @@
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
     </row>
-    <row r="43" ht="15.75" customHeight="1">
+    <row r="43" ht="13.5" customHeight="1">
       <c r="A43" s="8"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
@@ -1430,7 +1333,7 @@
       <c r="J43" s="8"/>
       <c r="K43" s="8"/>
     </row>
-    <row r="44" ht="15.75" customHeight="1">
+    <row r="44" ht="13.5" customHeight="1">
       <c r="A44" s="8"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
@@ -1443,7 +1346,7 @@
       <c r="J44" s="8"/>
       <c r="K44" s="8"/>
     </row>
-    <row r="45" ht="15.75" customHeight="1">
+    <row r="45" ht="13.5" customHeight="1">
       <c r="A45" s="8"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -1456,7 +1359,7 @@
       <c r="J45" s="8"/>
       <c r="K45" s="8"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1">
+    <row r="46" ht="13.5" customHeight="1">
       <c r="A46" s="8"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -1469,7 +1372,7 @@
       <c r="J46" s="8"/>
       <c r="K46" s="8"/>
     </row>
-    <row r="47" ht="15.75" customHeight="1">
+    <row r="47" ht="13.5" customHeight="1">
       <c r="A47" s="8"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
@@ -1482,7 +1385,7 @@
       <c r="J47" s="8"/>
       <c r="K47" s="8"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1">
+    <row r="48" ht="13.5" customHeight="1">
       <c r="A48" s="8"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
@@ -1495,7 +1398,7 @@
       <c r="J48" s="8"/>
       <c r="K48" s="8"/>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
+    <row r="49" ht="13.5" customHeight="1">
       <c r="A49" s="8"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
@@ -1508,7 +1411,7 @@
       <c r="J49" s="8"/>
       <c r="K49" s="8"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1">
+    <row r="50" ht="13.5" customHeight="1">
       <c r="A50" s="8"/>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
@@ -1521,7 +1424,7 @@
       <c r="J50" s="8"/>
       <c r="K50" s="8"/>
     </row>
-    <row r="51" ht="15.75" customHeight="1">
+    <row r="51" ht="13.5" customHeight="1">
       <c r="A51" s="8"/>
       <c r="B51" s="8"/>
       <c r="C51" s="8"/>
@@ -1534,7 +1437,7 @@
       <c r="J51" s="8"/>
       <c r="K51" s="8"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1">
+    <row r="52" ht="13.5" customHeight="1">
       <c r="A52" s="8"/>
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
@@ -1547,7 +1450,7 @@
       <c r="J52" s="8"/>
       <c r="K52" s="8"/>
     </row>
-    <row r="53" ht="15.75" customHeight="1">
+    <row r="53" ht="13.5" customHeight="1">
       <c r="A53" s="8"/>
       <c r="B53" s="8"/>
       <c r="C53" s="8"/>
@@ -1560,7 +1463,7 @@
       <c r="J53" s="8"/>
       <c r="K53" s="8"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1">
+    <row r="54" ht="13.5" customHeight="1">
       <c r="A54" s="8"/>
       <c r="B54" s="8"/>
       <c r="C54" s="8"/>
@@ -1573,7 +1476,7 @@
       <c r="J54" s="8"/>
       <c r="K54" s="8"/>
     </row>
-    <row r="55" ht="15.75" customHeight="1">
+    <row r="55" ht="13.5" customHeight="1">
       <c r="A55" s="8"/>
       <c r="B55" s="8"/>
       <c r="C55" s="8"/>
@@ -1586,7 +1489,7 @@
       <c r="J55" s="8"/>
       <c r="K55" s="8"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1">
+    <row r="56" ht="13.5" customHeight="1">
       <c r="A56" s="8"/>
       <c r="B56" s="8"/>
       <c r="C56" s="8"/>
@@ -1599,7 +1502,7 @@
       <c r="J56" s="8"/>
       <c r="K56" s="8"/>
     </row>
-    <row r="57" ht="15.75" customHeight="1">
+    <row r="57" ht="13.5" customHeight="1">
       <c r="A57" s="8"/>
       <c r="B57" s="8"/>
       <c r="C57" s="8"/>
@@ -1612,7 +1515,7 @@
       <c r="J57" s="8"/>
       <c r="K57" s="8"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1">
+    <row r="58" ht="13.5" customHeight="1">
       <c r="A58" s="8"/>
       <c r="B58" s="8"/>
       <c r="C58" s="8"/>
@@ -1625,7 +1528,7 @@
       <c r="J58" s="8"/>
       <c r="K58" s="8"/>
     </row>
-    <row r="59" ht="15.75" customHeight="1">
+    <row r="59" ht="13.5" customHeight="1">
       <c r="A59" s="8"/>
       <c r="B59" s="8"/>
       <c r="C59" s="8"/>
@@ -1638,7 +1541,7 @@
       <c r="J59" s="8"/>
       <c r="K59" s="8"/>
     </row>
-    <row r="60" ht="15.75" customHeight="1">
+    <row r="60" ht="13.5" customHeight="1">
       <c r="A60" s="8"/>
       <c r="B60" s="8"/>
       <c r="C60" s="8"/>
@@ -1651,7 +1554,7 @@
       <c r="J60" s="8"/>
       <c r="K60" s="8"/>
     </row>
-    <row r="61" ht="15.75" customHeight="1">
+    <row r="61" ht="13.5" customHeight="1">
       <c r="A61" s="8"/>
       <c r="B61" s="8"/>
       <c r="C61" s="8"/>
@@ -1664,7 +1567,7 @@
       <c r="J61" s="8"/>
       <c r="K61" s="8"/>
     </row>
-    <row r="62" ht="15.75" customHeight="1">
+    <row r="62" ht="13.5" customHeight="1">
       <c r="A62" s="8"/>
       <c r="B62" s="8"/>
       <c r="C62" s="8"/>
@@ -1677,7 +1580,7 @@
       <c r="J62" s="8"/>
       <c r="K62" s="8"/>
     </row>
-    <row r="63" ht="15.75" customHeight="1">
+    <row r="63" ht="13.5" customHeight="1">
       <c r="A63" s="8"/>
       <c r="B63" s="8"/>
       <c r="C63" s="8"/>
@@ -1690,7 +1593,7 @@
       <c r="J63" s="8"/>
       <c r="K63" s="8"/>
     </row>
-    <row r="64" ht="15.75" customHeight="1">
+    <row r="64" ht="13.5" customHeight="1">
       <c r="A64" s="8"/>
       <c r="B64" s="8"/>
       <c r="C64" s="8"/>
@@ -1703,7 +1606,7 @@
       <c r="J64" s="8"/>
       <c r="K64" s="8"/>
     </row>
-    <row r="65" ht="15.75" customHeight="1">
+    <row r="65" ht="13.5" customHeight="1">
       <c r="A65" s="8"/>
       <c r="B65" s="8"/>
       <c r="C65" s="8"/>
@@ -1716,7 +1619,7 @@
       <c r="J65" s="8"/>
       <c r="K65" s="8"/>
     </row>
-    <row r="66" ht="15.75" customHeight="1">
+    <row r="66" ht="13.5" customHeight="1">
       <c r="A66" s="8"/>
       <c r="B66" s="8"/>
       <c r="C66" s="8"/>
@@ -1729,7 +1632,7 @@
       <c r="J66" s="8"/>
       <c r="K66" s="8"/>
     </row>
-    <row r="67" ht="15.75" customHeight="1">
+    <row r="67" ht="13.5" customHeight="1">
       <c r="A67" s="8"/>
       <c r="B67" s="8"/>
       <c r="C67" s="8"/>
@@ -1742,7 +1645,7 @@
       <c r="J67" s="8"/>
       <c r="K67" s="8"/>
     </row>
-    <row r="68" ht="15.75" customHeight="1">
+    <row r="68" ht="13.5" customHeight="1">
       <c r="A68" s="8"/>
       <c r="B68" s="8"/>
       <c r="C68" s="8"/>
@@ -1755,7 +1658,7 @@
       <c r="J68" s="8"/>
       <c r="K68" s="8"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1">
+    <row r="69" ht="13.5" customHeight="1">
       <c r="A69" s="8"/>
       <c r="B69" s="8"/>
       <c r="C69" s="8"/>
@@ -1768,7 +1671,7 @@
       <c r="J69" s="8"/>
       <c r="K69" s="8"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1">
+    <row r="70" ht="13.5" customHeight="1">
       <c r="A70" s="8"/>
       <c r="B70" s="8"/>
       <c r="C70" s="8"/>
@@ -1781,7 +1684,7 @@
       <c r="J70" s="8"/>
       <c r="K70" s="8"/>
     </row>
-    <row r="71" ht="15.75" customHeight="1">
+    <row r="71" ht="13.5" customHeight="1">
       <c r="A71" s="8"/>
       <c r="B71" s="8"/>
       <c r="C71" s="8"/>
@@ -1794,7 +1697,7 @@
       <c r="J71" s="8"/>
       <c r="K71" s="8"/>
     </row>
-    <row r="72" ht="15.75" customHeight="1">
+    <row r="72" ht="13.5" customHeight="1">
       <c r="A72" s="8"/>
       <c r="B72" s="8"/>
       <c r="C72" s="8"/>
@@ -1807,7 +1710,7 @@
       <c r="J72" s="8"/>
       <c r="K72" s="8"/>
     </row>
-    <row r="73" ht="15.75" customHeight="1">
+    <row r="73" ht="13.5" customHeight="1">
       <c r="A73" s="8"/>
       <c r="B73" s="8"/>
       <c r="C73" s="8"/>
@@ -1820,7 +1723,7 @@
       <c r="J73" s="8"/>
       <c r="K73" s="8"/>
     </row>
-    <row r="74" ht="15.75" customHeight="1">
+    <row r="74" ht="13.5" customHeight="1">
       <c r="A74" s="8"/>
       <c r="B74" s="8"/>
       <c r="C74" s="8"/>
@@ -1833,7 +1736,7 @@
       <c r="J74" s="8"/>
       <c r="K74" s="8"/>
     </row>
-    <row r="75" ht="15.75" customHeight="1">
+    <row r="75" ht="13.5" customHeight="1">
       <c r="A75" s="8"/>
       <c r="B75" s="8"/>
       <c r="C75" s="8"/>
@@ -1846,7 +1749,7 @@
       <c r="J75" s="8"/>
       <c r="K75" s="8"/>
     </row>
-    <row r="76" ht="15.75" customHeight="1">
+    <row r="76" ht="13.5" customHeight="1">
       <c r="A76" s="8"/>
       <c r="B76" s="8"/>
       <c r="C76" s="8"/>
@@ -1859,7 +1762,7 @@
       <c r="J76" s="8"/>
       <c r="K76" s="8"/>
     </row>
-    <row r="77" ht="15.75" customHeight="1">
+    <row r="77" ht="13.5" customHeight="1">
       <c r="A77" s="8"/>
       <c r="B77" s="8"/>
       <c r="C77" s="8"/>
@@ -1872,7 +1775,7 @@
       <c r="J77" s="8"/>
       <c r="K77" s="8"/>
     </row>
-    <row r="78" ht="15.75" customHeight="1">
+    <row r="78" ht="13.5" customHeight="1">
       <c r="A78" s="8"/>
       <c r="B78" s="8"/>
       <c r="C78" s="8"/>
@@ -1885,7 +1788,7 @@
       <c r="J78" s="8"/>
       <c r="K78" s="8"/>
     </row>
-    <row r="79" ht="15.75" customHeight="1">
+    <row r="79" ht="13.5" customHeight="1">
       <c r="A79" s="8"/>
       <c r="B79" s="8"/>
       <c r="C79" s="8"/>
@@ -1898,7 +1801,7 @@
       <c r="J79" s="8"/>
       <c r="K79" s="8"/>
     </row>
-    <row r="80" ht="15.75" customHeight="1">
+    <row r="80" ht="13.5" customHeight="1">
       <c r="A80" s="8"/>
       <c r="B80" s="8"/>
       <c r="C80" s="8"/>
@@ -1911,7 +1814,7 @@
       <c r="J80" s="8"/>
       <c r="K80" s="8"/>
     </row>
-    <row r="81" ht="15.75" customHeight="1">
+    <row r="81" ht="13.5" customHeight="1">
       <c r="A81" s="8"/>
       <c r="B81" s="8"/>
       <c r="C81" s="8"/>
@@ -1924,7 +1827,7 @@
       <c r="J81" s="8"/>
       <c r="K81" s="8"/>
     </row>
-    <row r="82" ht="15.75" customHeight="1">
+    <row r="82" ht="13.5" customHeight="1">
       <c r="A82" s="8"/>
       <c r="B82" s="8"/>
       <c r="C82" s="8"/>
@@ -1937,7 +1840,7 @@
       <c r="J82" s="8"/>
       <c r="K82" s="8"/>
     </row>
-    <row r="83" ht="15.75" customHeight="1">
+    <row r="83" ht="13.5" customHeight="1">
       <c r="A83" s="8"/>
       <c r="B83" s="8"/>
       <c r="C83" s="8"/>
@@ -1950,7 +1853,7 @@
       <c r="J83" s="8"/>
       <c r="K83" s="8"/>
     </row>
-    <row r="84" ht="15.75" customHeight="1">
+    <row r="84" ht="13.5" customHeight="1">
       <c r="A84" s="8"/>
       <c r="B84" s="8"/>
       <c r="C84" s="8"/>
@@ -1963,7 +1866,7 @@
       <c r="J84" s="8"/>
       <c r="K84" s="8"/>
     </row>
-    <row r="85" ht="15.75" customHeight="1">
+    <row r="85" ht="13.5" customHeight="1">
       <c r="A85" s="8"/>
       <c r="B85" s="8"/>
       <c r="C85" s="8"/>
@@ -1976,7 +1879,7 @@
       <c r="J85" s="8"/>
       <c r="K85" s="8"/>
     </row>
-    <row r="86" ht="15.75" customHeight="1">
+    <row r="86" ht="13.5" customHeight="1">
       <c r="A86" s="8"/>
       <c r="B86" s="8"/>
       <c r="C86" s="8"/>
@@ -1989,7 +1892,7 @@
       <c r="J86" s="8"/>
       <c r="K86" s="8"/>
     </row>
-    <row r="87" ht="15.75" customHeight="1">
+    <row r="87" ht="13.5" customHeight="1">
       <c r="A87" s="8"/>
       <c r="B87" s="8"/>
       <c r="C87" s="8"/>
@@ -2002,7 +1905,7 @@
       <c r="J87" s="8"/>
       <c r="K87" s="8"/>
     </row>
-    <row r="88" ht="15.75" customHeight="1">
+    <row r="88" ht="13.5" customHeight="1">
       <c r="A88" s="8"/>
       <c r="B88" s="8"/>
       <c r="C88" s="8"/>
@@ -2015,7 +1918,7 @@
       <c r="J88" s="8"/>
       <c r="K88" s="8"/>
     </row>
-    <row r="89" ht="15.75" customHeight="1">
+    <row r="89" ht="13.5" customHeight="1">
       <c r="A89" s="8"/>
       <c r="B89" s="8"/>
       <c r="C89" s="8"/>
@@ -2028,7 +1931,7 @@
       <c r="J89" s="8"/>
       <c r="K89" s="8"/>
     </row>
-    <row r="90" ht="15.75" customHeight="1">
+    <row r="90" ht="13.5" customHeight="1">
       <c r="A90" s="8"/>
       <c r="B90" s="8"/>
       <c r="C90" s="8"/>
@@ -2041,7 +1944,7 @@
       <c r="J90" s="8"/>
       <c r="K90" s="8"/>
     </row>
-    <row r="91" ht="15.75" customHeight="1">
+    <row r="91" ht="13.5" customHeight="1">
       <c r="A91" s="8"/>
       <c r="B91" s="8"/>
       <c r="C91" s="8"/>
@@ -2054,7 +1957,7 @@
       <c r="J91" s="8"/>
       <c r="K91" s="8"/>
     </row>
-    <row r="92" ht="15.75" customHeight="1">
+    <row r="92" ht="13.5" customHeight="1">
       <c r="A92" s="8"/>
       <c r="B92" s="8"/>
       <c r="C92" s="8"/>
@@ -2067,7 +1970,7 @@
       <c r="J92" s="8"/>
       <c r="K92" s="8"/>
     </row>
-    <row r="93" ht="15.75" customHeight="1">
+    <row r="93" ht="13.5" customHeight="1">
       <c r="A93" s="8"/>
       <c r="B93" s="8"/>
       <c r="C93" s="8"/>
@@ -2080,7 +1983,7 @@
       <c r="J93" s="8"/>
       <c r="K93" s="8"/>
     </row>
-    <row r="94" ht="15.75" customHeight="1">
+    <row r="94" ht="13.5" customHeight="1">
       <c r="A94" s="8"/>
       <c r="B94" s="8"/>
       <c r="C94" s="8"/>
@@ -2093,7 +1996,7 @@
       <c r="J94" s="8"/>
       <c r="K94" s="8"/>
     </row>
-    <row r="95" ht="15.75" customHeight="1">
+    <row r="95" ht="13.5" customHeight="1">
       <c r="A95" s="8"/>
       <c r="B95" s="8"/>
       <c r="C95" s="8"/>
@@ -2106,7 +2009,7 @@
       <c r="J95" s="8"/>
       <c r="K95" s="8"/>
     </row>
-    <row r="96" ht="15.75" customHeight="1">
+    <row r="96" ht="13.5" customHeight="1">
       <c r="A96" s="8"/>
       <c r="B96" s="8"/>
       <c r="C96" s="8"/>
@@ -2119,7 +2022,7 @@
       <c r="J96" s="8"/>
       <c r="K96" s="8"/>
     </row>
-    <row r="97" ht="15.75" customHeight="1">
+    <row r="97" ht="13.5" customHeight="1">
       <c r="A97" s="8"/>
       <c r="B97" s="8"/>
       <c r="C97" s="8"/>
@@ -2132,7 +2035,7 @@
       <c r="J97" s="8"/>
       <c r="K97" s="8"/>
     </row>
-    <row r="98" ht="15.75" customHeight="1">
+    <row r="98" ht="13.5" customHeight="1">
       <c r="A98" s="8"/>
       <c r="B98" s="8"/>
       <c r="C98" s="8"/>
@@ -2145,7 +2048,7 @@
       <c r="J98" s="8"/>
       <c r="K98" s="8"/>
     </row>
-    <row r="99" ht="15.75" customHeight="1">
+    <row r="99" ht="13.5" customHeight="1">
       <c r="A99" s="8"/>
       <c r="B99" s="8"/>
       <c r="C99" s="8"/>
@@ -2158,7 +2061,7 @@
       <c r="J99" s="8"/>
       <c r="K99" s="8"/>
     </row>
-    <row r="100" ht="15.75" customHeight="1">
+    <row r="100" ht="13.5" customHeight="1">
       <c r="A100" s="8"/>
       <c r="B100" s="8"/>
       <c r="C100" s="8"/>
@@ -2173,44 +2076,44 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="C10:I10"/>
+    <mergeCell ref="C11:I11"/>
+    <mergeCell ref="C12:I12"/>
+    <mergeCell ref="C13:I13"/>
+    <mergeCell ref="A17:I30"/>
+    <mergeCell ref="A31:I33"/>
+    <mergeCell ref="A35:C39"/>
+    <mergeCell ref="D35:F39"/>
+    <mergeCell ref="C14:I14"/>
+    <mergeCell ref="C15:I15"/>
     <mergeCell ref="A16:I16"/>
-    <mergeCell ref="A17:I30"/>
-    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="A34:I34"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="D40:F40"/>
+    <mergeCell ref="G40:I40"/>
+    <mergeCell ref="G35:I39"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:G6"/>
     <mergeCell ref="A1:B4"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="H1:I8"/>
     <mergeCell ref="E1:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D40:F40"/>
-    <mergeCell ref="G40:I40"/>
-    <mergeCell ref="H1:I8"/>
-    <mergeCell ref="G35:I39"/>
-    <mergeCell ref="C12:I12"/>
-    <mergeCell ref="A9:I9"/>
-    <mergeCell ref="A31:I33"/>
-    <mergeCell ref="A34:I34"/>
-    <mergeCell ref="A35:C39"/>
-    <mergeCell ref="D35:F39"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C13:I13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:I14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C15:I15"/>
-    <mergeCell ref="C10:I10"/>
-    <mergeCell ref="C11:I11"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A7:B7"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>